<commit_message>
Publish B08 approved build
</commit_message>
<xml_diff>
--- a/downloads/exercises/basico-b08-b08-l05-practice-01.xlsx
+++ b/downloads/exercises/basico-b08-b08-l05-practice-01.xlsx
@@ -502,7 +502,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B11" s="25" t="str">
-        <x:v>Configura Comentario con longitud máxima de 30 caracteres y una alerta de Información.</x:v>
+        <x:v>Configura Fecha de entrega entre 01/09/2026 y 15/12/2026 y una alerta de Información.</x:v>
       </x:c>
       <x:c r="C11" s="23"/>
       <x:c r="D11" s="23"/>
@@ -598,7 +598,7 @@
         <x:v>Información</x:v>
       </x:c>
       <x:c r="B19" s="25" t="str">
-        <x:v>Comentario &gt; 30 caracteres</x:v>
+        <x:v>Fecha de entrega = 16/12/2026</x:v>
       </x:c>
       <x:c r="C19" s="25" t="str">
         <x:v>Informa; es la opción más flexible.</x:v>
@@ -821,7 +821,7 @@
         <x:v>Descuento</x:v>
       </x:c>
       <x:c r="E1" s="40" t="str">
-        <x:v>Comentario</x:v>
+        <x:v>Fecha de entrega</x:v>
       </x:c>
       <x:c r="F1" s="40" t="str">
         <x:v>Revisor</x:v>

</xml_diff>